<commit_message>
Resolve merge conflicts in calculations.py
</commit_message>
<xml_diff>
--- a/sample_data/Dwell time decay Worksheet Cylinder.xlsx
+++ b/sample_data/Dwell time decay Worksheet Cylinder.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\echorniak\GIT\BrachyD2ccEval\sample_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D937A7FD-CA04-472B-97D1-EC4376C7D0C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAC75CD7-8902-40D6-A88A-4066EEB3B23B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="35295" yWindow="1500" windowWidth="21600" windowHeight="12735" xr2:uid="{65AD33FA-F6BD-4A83-9802-8A1B68C48868}"/>
+    <workbookView xWindow="2730" yWindow="2730" windowWidth="21600" windowHeight="12645" xr2:uid="{65AD33FA-F6BD-4A83-9802-8A1B68C48868}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="Sheet2" sheetId="2" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$F$28</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$G$28</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Fraction Number</t>
   </si>
@@ -68,6 +68,9 @@
   </si>
   <si>
     <t>Total Time (sec):</t>
+  </si>
+  <si>
+    <t>Plan</t>
   </si>
 </sst>
 </file>
@@ -133,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -146,9 +149,6 @@
     <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -156,9 +156,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -542,7 +539,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F142A1C-31EE-496A-9657-8814021F0F9A}">
-  <dimension ref="A3:F29"/>
+  <dimension ref="A3:G29"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23.140625" customWidth="1"/>
@@ -550,87 +547,94 @@
     <col min="3" max="3" width="15.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="15.28515625" customWidth="1"/>
+    <col min="7" max="7" width="14.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:6" ht="36.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="4" spans="1:6" ht="40.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="11" t="s">
+    <row r="3" spans="1:7" ht="36.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="4" spans="1:7" ht="40.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="11"/>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-    </row>
-    <row r="5" spans="1:6" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+    </row>
+    <row r="5" spans="1:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B5" s="3"/>
     </row>
-    <row r="6" spans="1:6" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B6" s="3"/>
     </row>
-    <row r="7" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B7" s="3"/>
     </row>
-    <row r="9" spans="1:6" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B9" s="2">
+      <c r="B9" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" s="2">
         <v>1</v>
       </c>
-      <c r="C9" s="2">
+      <c r="D9" s="2">
         <v>2</v>
       </c>
-      <c r="D9" s="2">
+      <c r="E9" s="2">
         <v>3</v>
       </c>
-      <c r="E9" s="2">
+      <c r="F9" s="2">
         <v>4</v>
       </c>
-      <c r="F9" s="2">
+      <c r="G9" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="0.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" ht="0.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
-    </row>
-    <row r="11" spans="1:6" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G10" s="1"/>
+    </row>
+    <row r="11" spans="1:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B11" s="4"/>
+      <c r="B11" s="1"/>
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
       <c r="E11" s="4"/>
       <c r="F11" s="4"/>
-    </row>
-    <row r="12" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+      <c r="G11" s="4"/>
+    </row>
+    <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1"/>
-      <c r="B12" s="4"/>
+      <c r="B12" s="1"/>
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
       <c r="E12" s="4"/>
       <c r="F12" s="4"/>
-    </row>
-    <row r="13" spans="1:6" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G12" s="4"/>
+    </row>
+    <row r="13" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B13" s="5"/>
-      <c r="C13" s="6">
+      <c r="B13" s="1"/>
+      <c r="C13" s="5">
         <f>$B13*EXP((-1*LN(2)/73.81)*(C$11-$B$11))</f>
         <v>0</v>
       </c>
@@ -646,246 +650,265 @@
         <f>$B13*EXP((-1*LN(2)/73.81)*(F$11-$B$11))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" ht="0.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G13" s="6">
+        <f>$B13*EXP((-1*LN(2)/73.81)*(G$11-$B$11))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="0.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1"/>
-      <c r="B14" s="5"/>
-      <c r="C14" s="6">
-        <f>B14*EXP((-1*LN(2)/73.83)*(C$11-$B$11))</f>
-        <v>0</v>
-      </c>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-    </row>
-    <row r="15" spans="1:6" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B14" s="1"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="6">
+        <f>C14*EXP((-1*LN(2)/73.83)*(D$11-$C$11))</f>
+        <v>0</v>
+      </c>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="6"/>
+    </row>
+    <row r="15" spans="1:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B15" s="10">
-        <f>SUM(B17:B28)</f>
-        <v>0</v>
-      </c>
-      <c r="C15" s="10">
+      <c r="B15" s="1"/>
+      <c r="C15" s="8">
         <f>SUM(C17:C28)</f>
         <v>0</v>
       </c>
-      <c r="D15" s="10">
+      <c r="D15" s="8">
         <f>SUM(D17:D28)</f>
         <v>0</v>
       </c>
-      <c r="E15" s="10">
+      <c r="E15" s="8">
         <f>SUM(E17:E28)</f>
         <v>0</v>
       </c>
-      <c r="F15" s="10">
+      <c r="F15" s="8">
         <f>SUM(F17:F28)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G15" s="8">
+        <f>SUM(G17:G28)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B16" s="5"/>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B16" s="1"/>
+      <c r="C16" s="5"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="6"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
         <v>300</v>
       </c>
-      <c r="B17" s="8"/>
-      <c r="C17" s="9">
-        <f>$B17*EXP((LN(2)/73.81)*(C$11-$B$11))</f>
-        <v>0</v>
-      </c>
-      <c r="D17" s="9">
-        <f>$B17*EXP((LN(2)/73.81)*(D$11-$B$11))</f>
-        <v>0</v>
-      </c>
-      <c r="E17" s="9">
-        <f>$B17*EXP((LN(2)/73.81)*(E$11-$B$11))</f>
-        <v>0</v>
-      </c>
-      <c r="F17" s="9">
-        <f>$B17*EXP((LN(2)/73.81)*(F$11-$B$11))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B17" s="1"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="8">
+        <f>$C17*EXP((LN(2)/73.81)*(D$11-$C$11))</f>
+        <v>0</v>
+      </c>
+      <c r="E17" s="8">
+        <f>$C17*EXP((LN(2)/73.81)*(E$11-$C$11))</f>
+        <v>0</v>
+      </c>
+      <c r="F17" s="8">
+        <f>$C17*EXP((LN(2)/73.81)*(F$11-$C$11))</f>
+        <v>0</v>
+      </c>
+      <c r="G17" s="8">
+        <f>$C17*EXP((LN(2)/73.81)*(G$11-$C$11))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
         <v>295</v>
       </c>
-      <c r="B18" s="8"/>
-      <c r="C18" s="9">
-        <f t="shared" ref="C18:F22" si="0">$B18*EXP((LN(2)/73.81)*(C$11-$B$11))</f>
-        <v>0</v>
-      </c>
-      <c r="D18" s="9">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E18" s="9">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F18" s="9">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B18" s="1"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="8">
+        <f t="shared" ref="D18:G22" si="0">$C18*EXP((LN(2)/73.81)*(D$11-$C$11))</f>
+        <v>0</v>
+      </c>
+      <c r="E18" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F18" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G18" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
         <v>290</v>
       </c>
-      <c r="B19" s="8"/>
-      <c r="C19" s="9">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="D19" s="9">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E19" s="9">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F19" s="9">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B19" s="1"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E19" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F19" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G19" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
         <v>285</v>
       </c>
-      <c r="B20" s="8"/>
-      <c r="C20" s="9">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="D20" s="9">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E20" s="9">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F20" s="9">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B20" s="1"/>
+      <c r="C20" s="7"/>
+      <c r="D20" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E20" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F20" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G20" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
         <v>280</v>
       </c>
-      <c r="B21" s="8"/>
-      <c r="C21" s="9">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="D21" s="9">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E21" s="9">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F21" s="9">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B21" s="1"/>
+      <c r="C21" s="7"/>
+      <c r="D21" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E21" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F21" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G21" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
         <v>275</v>
       </c>
-      <c r="B22" s="8"/>
-      <c r="C22" s="9">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="D22" s="9">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E22" s="9">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F22" s="9">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B22" s="1"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E22" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F22" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G22" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
         <v>270</v>
       </c>
-      <c r="B23" s="8"/>
-      <c r="C23" s="9"/>
-      <c r="D23" s="9"/>
-      <c r="E23" s="9"/>
-      <c r="F23" s="9"/>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B23" s="1"/>
+      <c r="C23" s="7"/>
+      <c r="D23" s="8"/>
+      <c r="E23" s="8"/>
+      <c r="F23" s="8"/>
+      <c r="G23" s="8"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
         <v>265</v>
       </c>
-      <c r="B24" s="8"/>
-      <c r="C24" s="9"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="9"/>
-      <c r="F24" s="9"/>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B24" s="1"/>
+      <c r="C24" s="7"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="8"/>
+      <c r="G24" s="8"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
         <v>260</v>
       </c>
-      <c r="B25" s="8"/>
-      <c r="C25" s="9"/>
-      <c r="D25" s="9"/>
-      <c r="E25" s="9"/>
-      <c r="F25" s="9"/>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B25" s="1"/>
+      <c r="C25" s="7"/>
+      <c r="D25" s="8"/>
+      <c r="E25" s="8"/>
+      <c r="F25" s="8"/>
+      <c r="G25" s="8"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
         <v>255</v>
       </c>
-      <c r="B26" s="8"/>
-      <c r="C26" s="9"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="9"/>
-      <c r="F26" s="9"/>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B26" s="1"/>
+      <c r="C26" s="7"/>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="8"/>
+      <c r="G26" s="8"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
         <v>250</v>
       </c>
-      <c r="B27" s="8"/>
-      <c r="C27" s="9"/>
-      <c r="D27" s="9"/>
-      <c r="E27" s="9"/>
-      <c r="F27" s="9"/>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B27" s="1"/>
+      <c r="C27" s="7"/>
+      <c r="D27" s="8"/>
+      <c r="E27" s="8"/>
+      <c r="F27" s="8"/>
+      <c r="G27" s="8"/>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
         <v>245</v>
       </c>
-      <c r="B28" s="8"/>
-      <c r="C28" s="9"/>
-      <c r="D28" s="9"/>
-      <c r="E28" s="9"/>
-      <c r="F28" s="9"/>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B28" s="1"/>
+      <c r="C28" s="7"/>
+      <c r="D28" s="8"/>
+      <c r="E28" s="8"/>
+      <c r="F28" s="8"/>
+      <c r="G28" s="8"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>8</v>
       </c>

</xml_diff>